<commit_message>
Refactor disposal share arrays: Excel-driven, unified IS/noIS
- Deleted noIS_landfillShare[] and noIS_incinerationShare[] arrays
- Changed pw_landfillSharePerMat[] and pw_incinerationSharePerMat[] from
  hardcoded inline values to zero-init arrays loaded from Excel
- Added getCellNumericValue("Materials", row, 23/24) in Materials loop
- Both IS and noIS code paths now use same pw_* arrays
- Added pw_landfillShare (col W) and pw_incinerationShare (col X) to
  Materials sheet with orange highlighting; sum_check col Y verifies =1.0
- All 6 materials sum to 1.0; order matches AnyLogic matIndex()

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/20APRIL.xlsx
+++ b/20APRIL.xlsx
@@ -212,7 +212,7 @@
       <color rgb="001F497D"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -323,6 +323,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
         <bgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -490,7 +495,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -699,6 +704,9 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -7421,7 +7429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:Y8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="20" customWidth="1" style="67" min="1" max="1"/>
@@ -7559,6 +7567,21 @@
           <t>PricePaidToProvider_SGD_t</t>
         </is>
       </c>
+      <c r="W2" s="84" t="inlineStr">
+        <is>
+          <t>pw_landfillShare</t>
+        </is>
+      </c>
+      <c r="X2" s="84" t="inlineStr">
+        <is>
+          <t>pw_incinerationShare</t>
+        </is>
+      </c>
+      <c r="Y2" s="84" t="inlineStr">
+        <is>
+          <t>sum_check (must=1.0)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1" s="67">
       <c r="A3" t="inlineStr">
@@ -7634,6 +7657,16 @@
       <c r="V3" s="37" t="n">
         <v>-20</v>
       </c>
+      <c r="W3" s="85" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="X3" s="85" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="Y3" s="86">
+        <f>W3+X3</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="67">
       <c r="A4" t="inlineStr">
@@ -7709,6 +7742,16 @@
       <c r="V4" s="37" t="n">
         <v>-20</v>
       </c>
+      <c r="W4" s="85" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="X4" s="85" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Y4" s="86">
+        <f>W4+X4</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="67">
       <c r="A5" t="inlineStr">
@@ -7784,6 +7827,16 @@
       <c r="V5" s="37" t="n">
         <v>20</v>
       </c>
+      <c r="W5" s="85" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="X5" s="85" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="Y5" s="86">
+        <f>W5+X5</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="67">
       <c r="A6" t="inlineStr">
@@ -7859,6 +7912,16 @@
       <c r="V6" s="37" t="n">
         <v>-20</v>
       </c>
+      <c r="W6" s="85" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="X6" s="85" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="Y6" s="86">
+        <f>W6+X6</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="67">
       <c r="A7" t="inlineStr">
@@ -7934,6 +7997,16 @@
       <c r="V7" s="37" t="n">
         <v>20</v>
       </c>
+      <c r="W7" s="85" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="X7" s="85" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Y7" s="86">
+        <f>W7+X7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8008,6 +8081,16 @@
       </c>
       <c r="V8" s="37" t="n">
         <v>-5</v>
+      </c>
+      <c r="W8" s="85" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="X8" s="85" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="Y8" s="86">
+        <f>W8+X8</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -10236,8 +10319,8 @@
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B3:B5"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="B3:B5"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A18:A20"/>
   </mergeCells>

</xml_diff>